<commit_message>
Marcas madre Pispa, Nuara y Garra con fotos de empaque por marca
Cada registro lleva un producto de cada marca, sin nombres repetidos.
Pestaña Marcas por marca madre, fotos en tríptico y arreglo del zoom.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/salida/Productos_a_registrar_Guillermo.xlsx
+++ b/salida/Productos_a_registrar_Guillermo.xlsx
@@ -143,9 +143,9 @@
     <t>Septiembre 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Cortisol Support
-Cóctel de Calma
-Armonía Cortisol</t>
+    <t xml:space="preserve">Pispa Chill
+Nuara Armonía
+Garra Calm</t>
   </si>
   <si>
     <t>C6</t>
@@ -177,9 +177,9 @@
 • Beyond Vitamins Aguaje + Fenogreco 1000 mg (México): 1.313 u.</t>
   </si>
   <si>
-    <t xml:space="preserve">Aguaje Curvas
-Aguaje Amazónico
-Silueta Plena</t>
+    <t xml:space="preserve">Pispa Booty
+Nuara Silueta
+Garra Aguaje</t>
   </si>
   <si>
     <t>F65</t>
@@ -217,9 +217,9 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Feliz y Limpio
-Happy Cleaner
-Vientre Feliz</t>
+    <t xml:space="preserve">Pispa Detox
+Nuara Dicha
+Garra Limpio</t>
   </si>
   <si>
     <t>C2</t>
@@ -252,7 +252,9 @@
     <t>Últimos 28 días</t>
   </si>
   <si>
-    <t>Magnesio Kids</t>
+    <t xml:space="preserve">Pispa Kids Calm
+Nuara Cuento
+Garra Osito</t>
   </si>
   <si>
     <t>N6</t>
@@ -292,9 +294,9 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Gladiador
-Furia Espartana
-Elixir del Guerrero</t>
+    <t xml:space="preserve">Pispa Papi Shot
+Nuara Gladiador
+Garra Toro</t>
   </si>
   <si>
     <t>C4</t>
@@ -324,9 +326,9 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Genio Kids
-Mente Brillante Kids
-Estrellitas de Atención</t>
+    <t xml:space="preserve">Pispa Kids Focus
+Nuara Foco
+Garra Junior</t>
   </si>
   <si>
     <t>C5</t>
@@ -351,9 +353,9 @@
     <t>• Bcuelov Cayenne Pepper Supplement (EE. UU.):  u.</t>
   </si>
   <si>
-    <t xml:space="preserve">Cayena Térmica
-Fuego Natural
-Metabolismo Activo</t>
+    <t xml:space="preserve">Pispa Picante
+Nuara Cayena
+Garra Fuego</t>
   </si>
   <si>
     <t>F39</t>
@@ -387,9 +389,9 @@
 • k2o Advanced Skin Hydration Mix (EE. UU.): 6.716 u.</t>
   </si>
   <si>
-    <t xml:space="preserve">Colágeno Firmeza Total
-Seda Marina
-Rodillas Sanas</t>
+    <t xml:space="preserve">Pispa Glow Shake
+Nuara Piel
+Garra Flex</t>
   </si>
   <si>
     <t>F06</t>
@@ -424,9 +426,9 @@
 • NUTRAHARMONY Biotin Gummies Sugar (EE. UU.): 515 u.</t>
   </si>
   <si>
-    <t xml:space="preserve">Cabello Fuerte
-Biotina Brillante
-Melena Sana</t>
+    <t xml:space="preserve">Pispa Melena
+Nuara Cabellera
+Garra Tupido</t>
   </si>
   <si>
     <t>N4</t>
@@ -455,9 +457,9 @@
 • Lemme Sleep Gummies with 5mg Melatonin, Magnesium, L (EE. UU.): 1.300 u.</t>
   </si>
   <si>
-    <t xml:space="preserve">Noche Plena
-Sueño Dulce
-Melatonina Serena</t>
+    <t xml:space="preserve">Pispa Sleep
+Nuara Sueño
+Garra Noche</t>
   </si>
   <si>
     <t>N1</t>
@@ -484,9 +486,9 @@
 • First Day Kids Calming Magnesium Gummies Ages 4 (EE. UU.): 288 u.</t>
   </si>
   <si>
-    <t xml:space="preserve">Gotitas de Calma
-Magnesio Infantil
-Pequeño Sereno</t>
+    <t xml:space="preserve">Pispa Kids Calm Gotas
+Nuara Nana
+Garra Mini</t>
   </si>
   <si>
     <t>N5</t>
@@ -520,9 +522,9 @@
 • Gardenika Organic Laxative Loose Leaf Tea, Caffeine (EE. UU.): 15 u.</t>
   </si>
   <si>
-    <t xml:space="preserve">Té Vientre Libre
-Hoja de Sen
-Té Despeje</t>
+    <t xml:space="preserve">Pispa Fluye Té
+Nuara Alivio
+Garra Libre</t>
   </si>
   <si>
     <t>N3</t>
@@ -550,9 +552,9 @@
 • $1 AUCTIONS Soursop Sleep Drops with Melatonin 5mg, Ashwagandha &amp; L (EE. UU.): 13 u.</t>
   </si>
   <si>
-    <t xml:space="preserve">Gotas de Sueño
-Luna Líquida
-Descanso Rápido</t>
+    <t xml:space="preserve">Pispa Sleep Gotas
+Nuara Luna
+Garra Off</t>
   </si>
   <si>
     <t>N2</t>
@@ -576,9 +578,9 @@
 • UPMER Pack Magnesio 7 en 1 + Omega 3 (México): 3.051 u.</t>
   </si>
   <si>
-    <t xml:space="preserve">Magnesio Reparador
-Reposo Profundo
-Piernas en Calma</t>
+    <t xml:space="preserve">Pispa Magnesio
+Nuara Reposo
+Garra Mag</t>
   </si>
   <si>
     <t>F01</t>
@@ -608,9 +610,9 @@
 • Vital Source Feminine Balance Gummies (EE. UU.): 10.985 u.</t>
   </si>
   <si>
-    <t xml:space="preserve">Equilibrio Íntimo
-Pétalo Íntimo
-Frescura Femenina</t>
+    <t xml:space="preserve">Pispa Miau
+Nuara Íntima
+Garra Flora</t>
   </si>
   <si>
     <t>F02</t>
@@ -630,9 +632,9 @@
 • LeeFar Cutting Drops Lymphatic Debloat (EE. UU.): 15.488 u.</t>
   </si>
   <si>
-    <t xml:space="preserve">Gotas Drenantes
-Manantial Depurativo
-Piernas Livianas</t>
+    <t xml:space="preserve">Pispa Drena Gotas
+Nuara Fluida
+Garra Desinfla Gotas</t>
   </si>
   <si>
     <t>F09</t>
@@ -659,9 +661,9 @@
 • NeoCell Creatine Monohydrate + Multi Collagen (EE. UU.): 11.436 u.</t>
   </si>
   <si>
-    <t xml:space="preserve">Glúteo Activo
-Silueta Esculpida
-Curvas de Mujer</t>
+    <t xml:space="preserve">Pispa Power
+Nuara Curva
+Garra Glute</t>
   </si>
   <si>
     <t>F04</t>
@@ -685,9 +687,9 @@
 • Windboss Hack your Tummy (paquete) (México): 14.245 u.</t>
   </si>
   <si>
-    <t xml:space="preserve">Digestión Ligera
-Jardín Intestinal
-Vientre Sereno</t>
+    <t xml:space="preserve">Pispa Pancita
+Nuara Ligera
+Garra Gut</t>
   </si>
   <si>
     <t>F03</t>
@@ -708,9 +710,9 @@
 • HS Hero Sport Creatina Monohidratada 650 g (México): 1.209 u.</t>
   </si>
   <si>
-    <t xml:space="preserve">Creatina Fuerza Real
-Roble Atlético
-Músculo Firme</t>
+    <t xml:space="preserve">Pispa Power Pura
+Nuara Fuerza
+Garra Crea</t>
   </si>
   <si>
     <t>F05</t>
@@ -730,9 +732,9 @@
 • Toplux Organic Beet Root Capsules (EE. UU.): 18.180 u.</t>
   </si>
   <si>
-    <t xml:space="preserve">Potencia Circulatoria
-Raíz Roja Vital
-Hombre Vigoroso</t>
+    <t xml:space="preserve">Pispa Firme
+Nuara Vigor
+Garra Pump</t>
   </si>
   <si>
     <t>F11</t>
@@ -768,9 +770,9 @@
 • Toyocare Bebida relajante Ashwagandha KSM-66 (México): 1.565 u.</t>
   </si>
   <si>
-    <t xml:space="preserve">Bebida Relajante Nocturna
-Tisana de Luna
-Noche Tranquila</t>
+    <t xml:space="preserve">Pispa Relax
+Nuara Ocaso
+Garra Chill</t>
   </si>
   <si>
     <t>F07</t>
@@ -796,9 +798,9 @@
 • SWIYIE Complejo de Colágeno Múltiple (120 cápsulas) (México): 6.545 u.</t>
   </si>
   <si>
-    <t xml:space="preserve">Colágeno Belleza Integral
-Esencia de Perla
-Mujer Radiante</t>
+    <t xml:space="preserve">Pispa Glow
+Nuara Lozana
+Garra Piel</t>
   </si>
   <si>
     <t>F08</t>
@@ -816,9 +818,9 @@
     <t>• Vitafusion Fiber Well Sugar Free Gummies (EE. UU.): 38.736 u.</t>
   </si>
   <si>
-    <t xml:space="preserve">Gomitas de Fibra Diaria
-Fibra Suave
-Tránsito Ligero</t>
+    <t xml:space="preserve">Pispa Fluye
+Nuara Ritmo
+Garra Fibra</t>
   </si>
   <si>
     <t>F40</t>
@@ -844,9 +846,9 @@
 • VEV DeepCalm Magnesium Complex Gummies 14-in-1 (EE. UU.): 18.378 u.</t>
   </si>
   <si>
-    <t xml:space="preserve">Gomas Sueño Profundo
-Sueño de Algodón
-Dulces Sueños</t>
+    <t xml:space="preserve">Pispa Mimir
+Nuara Arrullo
+Garra Rest</t>
   </si>
   <si>
     <t>F16</t>
@@ -867,9 +869,9 @@
     <t>• Toplux Organic Beet Root Tablets 2040mg (EE. UU.): 22.673 u.</t>
   </si>
   <si>
-    <t xml:space="preserve">Remolacha Roja Pura
-Raíz Carmesí
-Presión Serena</t>
+    <t xml:space="preserve">Pispa Red Tabs
+Nuara Pulso
+Garra Bombeo</t>
   </si>
   <si>
     <t>F35</t>
@@ -891,9 +893,9 @@
     <t>• Windboss Combo Cortisol + Myo-Inositol (kit 2 frascos) (México): 28.383 u.</t>
   </si>
   <si>
-    <t xml:space="preserve">Control de Cortisol
-Armonía Hormonal
-Vientre sin Estrés</t>
+    <t xml:space="preserve">Pispa Cortisol
+Nuara Calma
+Garra Temple</t>
   </si>
   <si>
     <t>F14</t>
@@ -911,9 +913,9 @@
     <t>• Body Magic Chlorophyll Pill (EE. UU.): 19.913 u.</t>
   </si>
   <si>
-    <t xml:space="preserve">Clorofila Sin Olor
-Frescura Verde
-Cuerpo Fresco</t>
+    <t xml:space="preserve">Pispa Fresh
+Nuara Fresca
+Garra Verde</t>
   </si>
   <si>
     <t>F72</t>
@@ -944,9 +946,9 @@
 • Windboss Cápsulas de Vitalidad y Resistencia 2026 (México): 1.588 u.</t>
   </si>
   <si>
-    <t xml:space="preserve">Vigor Masculino
-Potencia Andina
-Hombre de Hierro</t>
+    <t xml:space="preserve">Pispa Papi
+Nuara Potencia
+Garra Rey</t>
   </si>
   <si>
     <t>F24</t>
@@ -1025,9 +1027,9 @@
     <t>• YESNAP Lymphatic Drainage Support 12-in-1 (30 sticks, naranja-mango) (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Drenaje Linfático Express
-Doce Plantas
-Cuerpo Ligero</t>
+    <t xml:space="preserve">Pispa Drena Stick
+Nuara Cauce
+Garra Seco</t>
   </si>
   <si>
     <t>F27</t>
@@ -1047,9 +1049,9 @@
 • Micro Ingredients Oregano Oil with Black Seed Oil (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Orégano y Semilla Negra
-Semilla Negra Ancestral
-Escudo Natural</t>
+    <t xml:space="preserve">Pispa Orégano
+Nuara Guardiana
+Garra Escudo</t>
   </si>
   <si>
     <t>F76</t>
@@ -1067,9 +1069,9 @@
     <t>• Bella All Natural Colon Cleanse 400g (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Colon Limpio Papaya
-Hoja de Papaya
-Vientre en Paz</t>
+    <t xml:space="preserve">Pispa Papaya
+Nuara Limpia
+Garra Reset</t>
   </si>
   <si>
     <t>F80</t>
@@ -1087,9 +1089,9 @@
     <t>• Nutricost NAC N-Acetyl L-Cysteine Capsules (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">NAC Depura
-Hígado Puro
-Respiro Limpio</t>
+    <t xml:space="preserve">Pispa Respira
+Nuara Respiro
+Garra Filtro</t>
   </si>
   <si>
     <t>F77</t>
@@ -1110,9 +1112,9 @@
     <t>• Milamiamor 15 Day Cleanse (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Limpieza 15 Días
-Depuración Herbal
-Ligereza Total</t>
+    <t xml:space="preserve">Pispa Reset
+Nuara Reinicio
+Garra Purga</t>
   </si>
   <si>
     <t>F50</t>
@@ -1139,9 +1141,9 @@
     <t>• ATRAKT D-BLOAT Advanced Debloat Powder (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Vientre Desinflamado
-Botánica Depurativa
-Adiós Hinchazón</t>
+    <t xml:space="preserve">Pispa Planita
+Nuara Vientre
+Garra Flat</t>
   </si>
   <si>
     <t>F31</t>
@@ -1160,9 +1162,9 @@
     <t>• BioGaia Fresh Breath Oral Probiotics (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Aliento Fresco Diario
-Boca Equilibrada
-Sonrisa Segura</t>
+    <t xml:space="preserve">Pispa Besito
+Nuara Aliento
+Garra Fresh</t>
   </si>
   <si>
     <t>F73</t>
@@ -1180,9 +1182,9 @@
     <t>• Horbäach Liquid Chlorophyll Drops (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Gotas de Clorofila
-Hoja Viva
-Agua Verde</t>
+    <t xml:space="preserve">Pispa Fresh Gotas
+Nuara Rocío
+Garra Verde Gotas</t>
   </si>
   <si>
     <t>F33</t>
@@ -1198,9 +1200,9 @@
 • MVPCARE Desintoxicación Linfática (México)</t>
   </si>
   <si>
-    <t xml:space="preserve">Drenaje Linfático Total
-Jardín Depurativo
-Menos Retención</t>
+    <t xml:space="preserve">Pispa Drena
+Nuara Liviana
+Garra Desinfla</t>
   </si>
   <si>
     <t xml:space="preserve">• LeafLea Senna Tea Bags (EE. UU.)
@@ -1261,9 +1263,9 @@
     <t>• Loosey Goosey Calming Pouches 3 Pack (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Bolsitas Calma
-Kava Serena
-Pausa Serena</t>
+    <t xml:space="preserve">Pispa Calma
+Nuara Pausa
+Garra Frío</t>
   </si>
   <si>
     <t>F43</t>
@@ -1288,9 +1290,9 @@
     <t>• Windboss Ashwagandha KSM-66 + L-Teanina + PS (México)</t>
   </si>
   <si>
-    <t xml:space="preserve">Cortisol en Calma
-Raíz de Calma
-Mente Tranquila</t>
+    <t xml:space="preserve">Pispa Zen
+Nuara Sosiego
+Garra Aplomo</t>
   </si>
   <si>
     <t xml:space="preserve">• Project Superhuman DreamOn Sleep Gummies for Adult Men &amp; Women, 8 (EE. UU.)
@@ -1346,9 +1348,9 @@
 • Wellah Electrolytes Sample Pack + Shaker (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Hidratación Inmediata
-Brisa Mineral
-Suero Recuperador</t>
+    <t xml:space="preserve">Pispa Suero
+Nuara Oasis
+Garra Hidra</t>
   </si>
   <si>
     <t>F68</t>
@@ -1371,9 +1373,9 @@
 • Windboss NAD+ Liposomal NR 900 mg (100 cápsulas) (México)</t>
   </si>
   <si>
-    <t xml:space="preserve">NAD+ Celular
-Longevidad Activa
-Energía de Juventud</t>
+    <t xml:space="preserve">Pispa Young
+Nuara Longeva
+Garra Cell</t>
   </si>
   <si>
     <t>F20</t>
@@ -1399,9 +1401,9 @@
 • Montue Gotitas B12 + B6 (40 porciones, frambuesa) (México)</t>
   </si>
   <si>
-    <t xml:space="preserve">Complejo B Energía
-Claridad Andina
-Energía Constante</t>
+    <t xml:space="preserve">Pispa Pila
+Nuara Despierta
+Garra Boost</t>
   </si>
   <si>
     <t>F28</t>
@@ -1417,9 +1419,9 @@
 • Vital Source Creatine Gummies (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Creatina Masticable
-Fuerza Pura
-Rendimiento Diario</t>
+    <t xml:space="preserve">Pispa Power Gummies
+Nuara Tono
+Garra Crea Gum</t>
   </si>
   <si>
     <t>F22</t>
@@ -1437,9 +1439,9 @@
     <t>• BODYHEALTH Perfect Amino Tablets (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Músculo Esencial
-Ocho Esenciales
-Recuperación Activa</t>
+    <t xml:space="preserve">Pispa Amino
+Nuara Esencial
+Garra Recarga</t>
   </si>
   <si>
     <t>F23</t>
@@ -1461,9 +1463,9 @@
 • Euphoric 100% Whey Protein + Creatina (México)</t>
   </si>
   <si>
-    <t xml:space="preserve">Proteína con Colágeno
-Suero Dorado
-Batido Atleta</t>
+    <t xml:space="preserve">Pispa Protein
+Nuara Esculpida
+Garra Whey</t>
   </si>
   <si>
     <t>F69</t>
@@ -1478,9 +1480,9 @@
     <t>• Cata-Kor NMN Powder 1000 mg (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">NMN Polvo Puro
-Origen Celular
-Juventud Diaria</t>
+    <t xml:space="preserve">Pispa Young Drink
+Nuara Aurora
+Garra Motor</t>
   </si>
   <si>
     <t>F59</t>
@@ -1500,9 +1502,9 @@
     <t>• Toyocare palitos de miel con shilajit (30 unidades) (México)</t>
   </si>
   <si>
-    <t xml:space="preserve">Miel con Shilajit
-Néctar Negro
-Miel Potente</t>
+    <t xml:space="preserve">Pispa Honey
+Nuara Brío
+Garra Roca</t>
   </si>
   <si>
     <t>Salud íntima y libido femenina  ·  6 registros</t>
@@ -1535,9 +1537,9 @@
 • VivoNu Probióticos para la Mujer con Arándano (México)</t>
   </si>
   <si>
-    <t xml:space="preserve">Equilibrio Femenino
-Arándano Íntimo
-Mujer Protegida</t>
+    <t xml:space="preserve">Pispa Arándano
+Nuara Flora
+Garra Berry</t>
   </si>
   <si>
     <t>F63</t>
@@ -1562,9 +1564,9 @@
     <t>• Adapto Drive Maca Root Drops (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Gotas del Deseo
-Raíz del Deseo
-Pasión Diaria</t>
+    <t xml:space="preserve">Pispa Fuego
+Nuara Deseo
+Garra Ganas</t>
   </si>
   <si>
     <t>F45</t>
@@ -1587,9 +1589,9 @@
     <t>• Nello Superbalance Hormonal Support Drink Mix (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Súper Balance Hormonal
-Luna Botánica
-Equilibrio Mensual</t>
+    <t xml:space="preserve">Pispa Balance
+Nuara Equilibrio
+Garra Ella</t>
   </si>
   <si>
     <t>F44</t>
@@ -1609,9 +1611,9 @@
 • Zesty Pro Inositol 200 g + Pink Fury 100 g (México)</t>
   </si>
   <si>
-    <t xml:space="preserve">Ciclo Regular
-Armonía Ovárica
-Fertilidad Plena</t>
+    <t xml:space="preserve">Pispa Hormonita
+Nuara Ciclo
+Garra Ritmo</t>
   </si>
   <si>
     <t>F64</t>
@@ -1631,9 +1633,9 @@
     <t>• Montue Maca &amp; Fenogreco Gummies Combo (México)</t>
   </si>
   <si>
-    <t xml:space="preserve">Gomitas Curvas Plenas
-Maca Florecer
-Curvas y Deseo</t>
+    <t xml:space="preserve">Pispa Curvas
+Nuara Diosa
+Garra Curva</t>
   </si>
   <si>
     <t>Quemar grasa y bajar de peso  ·  8 registros</t>
@@ -1660,9 +1662,9 @@
     <t>• Apothékary Blue Burn Metabolic Support Drops (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Gotas Sin Antojos
-Fuego Azul
-Metabolismo en Marcha</t>
+    <t xml:space="preserve">Pispa Slim Gotas
+Nuara Templanza
+Garra Cut</t>
   </si>
   <si>
     <t>F79</t>
@@ -1683,9 +1685,9 @@
     <t>• Coleology Cutting Jelly (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Jalea Saciante
-Jalea Silueta
-Cintura Fina</t>
+    <t xml:space="preserve">Pispa Jelly
+Nuara Saciada
+Garra Full</t>
   </si>
   <si>
     <t>F34</t>
@@ -1704,9 +1706,9 @@
     <t>• Yesnap MOCKTALE-1 Metabolic Drink Mix (30 sobres) (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Control de Antojos
-Berberina Esbelta
-Saciedad Natural</t>
+    <t xml:space="preserve">Pispa Slim
+Nuara Mesura
+Garra Lean</t>
   </si>
   <si>
     <t>F42</t>
@@ -1729,9 +1731,9 @@
     <t>• Blood Sugar Complex 20 Vitamins &amp; Minerals (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Glucosa Estable
-Canela y Gymnema
-Azúcar en Balance</t>
+    <t xml:space="preserve">Pispa Glucosa
+Nuara Balance
+Garra Nivel</t>
   </si>
   <si>
     <t>F13</t>
@@ -1754,9 +1756,9 @@
 • Multiblue Berberina HCl con Canela y Cúrcuma (México)</t>
   </si>
   <si>
-    <t xml:space="preserve">Berberina Equilibrio Azúcar
-Raíz Dorada
-Azúcar en Orden</t>
+    <t xml:space="preserve">Pispa Berberina
+Nuara Esbelta
+Garra Freno</t>
   </si>
   <si>
     <t>F10</t>
@@ -1785,9 +1787,9 @@
     <t>• Leefar Cutting Bundle (Cutting Mix + Cutting Drops) (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Berberina Termogénica
-Silueta Botánica
-Una Talla Menos</t>
+    <t xml:space="preserve">Pispa Burn Drink
+Nuara Contorno
+Garra Shred</t>
   </si>
   <si>
     <t>F41</t>
@@ -1808,9 +1810,9 @@
     <t>• Toplux Keto Burn (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Quemador Keto Total
-Mango y Frambuesa
-Cintura Definida</t>
+    <t xml:space="preserve">Pispa Burn
+Nuara Brasa
+Garra Quema</t>
   </si>
   <si>
     <t>F12</t>
@@ -1832,9 +1834,9 @@
     <t>• Montue Gomitas de ACV (México)</t>
   </si>
   <si>
-    <t xml:space="preserve">Vinagre Adelgazante
-Manzana Dorada
-Sin Antojos</t>
+    <t xml:space="preserve">Pispa Manzanita
+Nuara Manzana
+Garra Apple</t>
   </si>
   <si>
     <t>Colágeno y antiedad  ·  7 registros</t>
@@ -1861,9 +1863,9 @@
     <t>• Cymbiotika Liposomal Glutathione (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Glutatión Luminoso
-Piel de Porcelana
-Tono Uniforme</t>
+    <t xml:space="preserve">Pispa Bright Shot
+Nuara Luz
+Garra Glow</t>
   </si>
   <si>
     <t>F25</t>
@@ -1886,9 +1888,9 @@
 • Cata-Kor Liposomal Glutathione 1155 mg (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Glutatión Radiante
-Piel Luminosa
-Tono Parejo</t>
+    <t xml:space="preserve">Pispa Bright
+Nuara Luminosa
+Garra Parejo</t>
   </si>
   <si>
     <t>F51</t>
@@ -1903,9 +1905,9 @@
     <t>• Youtheory Collagen Liquid 5,000 mg (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Colágeno Líquido Total
-Piel de Nácar
-Firmeza Diaria</t>
+    <t xml:space="preserve">Pispa Glow Shot
+Nuara Firme
+Garra Joint</t>
   </si>
   <si>
     <t>F71</t>
@@ -1923,9 +1925,9 @@
     <t>• Micro Ingredients Astaxanthin 12mg (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Astaxantina Marina
-Microalga Roja
-Escudo Juvenil</t>
+    <t xml:space="preserve">Pispa Pink
+Nuara Tersa
+Garra Rojo</t>
   </si>
   <si>
     <t>F70</t>
@@ -1944,9 +1946,9 @@
     <t>• Megneta NAD+ Resveratrol 1200 mg Liposomal (México)</t>
   </si>
   <si>
-    <t xml:space="preserve">NAD+ Resveratrol
-Uva Longeva
-Tiempo Detenido</t>
+    <t xml:space="preserve">Pispa Forever
+Nuara Atemporal
+Garra Tiempo</t>
   </si>
   <si>
     <t xml:space="preserve">• Péptidos de colágeno bovino tipo I y III 10-20 g por porción, o multi-tipo (I, II, III, V, X)
@@ -1987,9 +1989,9 @@
     <t>• Horbäach Nitric Oxide Beet Root Gummies (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Gomitas de Remolacha
-Corazón Rojo
-Pulso Vital</t>
+    <t xml:space="preserve">Pispa Red Gummies
+Nuara Rubí
+Garra Beet Gum</t>
   </si>
   <si>
     <t>F48</t>
@@ -2008,9 +2010,9 @@
 • B Life Omega 3 Aceite de Salmón (México)</t>
   </si>
   <si>
-    <t xml:space="preserve">Omega Corazón
-Mar Antártico
-Memoria y Corazón</t>
+    <t xml:space="preserve">Pispa Omega
+Nuara Marina
+Garra Ancla</t>
   </si>
   <si>
     <t>F38</t>
@@ -2034,9 +2036,9 @@
     <t>• VivoNu Cayenne Pepper Softgels (México)</t>
   </si>
   <si>
-    <t xml:space="preserve">Corazón Fuerte
-Espino Real
-Circulación Total</t>
+    <t xml:space="preserve">Pispa Heart
+Nuara Corazón
+Garra Latido</t>
   </si>
   <si>
     <t>F37</t>
@@ -2054,9 +2056,9 @@
     <t>• NEWELLME Beetroot Super Red Food Powder (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Remolacha en Polvo Activa
-Cosecha Roja
-Rendimiento Rojo</t>
+    <t xml:space="preserve">Pispa Red
+Nuara Torrente
+Garra Beet</t>
   </si>
   <si>
     <t>Defensas y vitaminas  ·  7 registros</t>
@@ -2080,9 +2082,9 @@
     <t>• Bella All Natural D3 K2 Drops Omega 3 MCT (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Gotas de Sol
-Sol Líquido
-Defensa Familiar</t>
+    <t xml:space="preserve">Pispa Sol Gotas
+Nuara Sol
+Garra Base</t>
   </si>
   <si>
     <t>F74</t>
@@ -2106,9 +2108,9 @@
     <t>• Hrvsta 20-Herb Blend Capsules (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Musgo Marino Veinte
-Veinte Hierbas
-Escudo Herbal</t>
+    <t xml:space="preserve">Pispa Sea Moss
+Nuara Escudo
+Garra Musgo</t>
   </si>
   <si>
     <t>F15</t>
@@ -2125,9 +2127,9 @@
 • Toyocare Vitamina D3 + K2 10.000 IU (México)</t>
   </si>
   <si>
-    <t xml:space="preserve">Hueso Fuerte D3+K2
-Luz Mediterránea
-Sol en Cápsula</t>
+    <t xml:space="preserve">Pispa Sol
+Nuara Solar
+Garra Rayo</t>
   </si>
   <si>
     <t>F54</t>
@@ -2146,9 +2148,9 @@
     <t>• Santa Cruz Paleo Zinc + Copper Caps (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Zinc y Cobre
-Mineral Ancestral
-Escudo Mineral</t>
+    <t xml:space="preserve">Pispa Zinc
+Nuara Cobre
+Garra Metal</t>
   </si>
   <si>
     <t>F56</t>
@@ -2169,9 +2171,9 @@
     <t>• Nature Made GLP-1 Companion Health Pack (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Compañero GLP-1
-Nutrición Consciente
-Respaldo Diario</t>
+    <t xml:space="preserve">Pispa Slim Care
+Nuara Compañera
+Garra Aliado</t>
   </si>
   <si>
     <t>F26</t>
@@ -2189,9 +2191,9 @@
     <t>• Toplux Moringa Capsules 1200mg (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Moringa Vital
-Hoja Verde Pura
-Energía del Campo</t>
+    <t xml:space="preserve">Pispa Green
+Nuara Verdor
+Garra Hoja</t>
   </si>
   <si>
     <t>F55</t>
@@ -2212,9 +2214,9 @@
     <t>• Rainbow Light Men's Multivitamin (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Hombre Activo
-Vitalidad Noble
-Energía Varonil</t>
+    <t xml:space="preserve">Pispa Man
+Nuara Hombre
+Garra Diario</t>
   </si>
   <si>
     <t>Cabello, piel y uñas  ·  6 registros</t>
@@ -2242,9 +2244,9 @@
 • MaryRuth's Daily Liquid Hair Formula (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Biotina Líquida Capilar
-Cabellera de Seda
-Melena Larga</t>
+    <t xml:space="preserve">Pispa Melena Drops
+Nuara Cascada
+Garra Crece</t>
   </si>
   <si>
     <t>F21</t>
@@ -2265,9 +2267,9 @@
     <t>• Bears with Benefits Biotin Gummies (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Gomitas Belleza Completa
-Jardín de Belleza
-Belleza Diaria</t>
+    <t xml:space="preserve">Pispa Glow Gummies
+Nuara Radiante
+Garra Facha</t>
   </si>
   <si>
     <t xml:space="preserve">• Bears with Benefits Biotin Gummies (EE. UU.)
@@ -2296,9 +2298,9 @@
     <t>• Clear Skin Acne Supplement (Clear-3) (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Piel Despejada
-Pureza Dérmica
-Cara Limpia</t>
+    <t xml:space="preserve">Pispa Clear
+Nuara Pura
+Garra Poro</t>
   </si>
   <si>
     <t>F52</t>
@@ -2319,9 +2321,9 @@
 • Josend MaxBiotin MultiVita (México)</t>
   </si>
   <si>
-    <t xml:space="preserve">Biotina Triple Belleza
-Seda Natural
-Melena Fuerte</t>
+    <t xml:space="preserve">Pispa Beauty
+Nuara Esplendor
+Garra Pinta</t>
   </si>
   <si>
     <t>F19</t>
@@ -2338,9 +2340,9 @@
     <t>• Megneta Complejo Avanzado Crecimiento del Cabello (México)</t>
   </si>
   <si>
-    <t xml:space="preserve">Fórmula Anticaída
-Bosque Capilar
-Cabello Abundante</t>
+    <t xml:space="preserve">Pispa Melena Max
+Nuara Raíz
+Garra Brote</t>
   </si>
   <si>
     <t>Potencia sexual masculina  ·  4 registros</t>
@@ -2371,9 +2373,9 @@
     <t>• Moshe Vitalidad Masculina 5 Tesoros (México)</t>
   </si>
   <si>
-    <t xml:space="preserve">Té Vigor Masculino
-Cinco Tesoros
-Hierro Varonil</t>
+    <t xml:space="preserve">Pispa Papi Té
+Nuara Tesoro
+Garra Cinco</t>
   </si>
   <si>
     <t>F58</t>
@@ -2395,9 +2397,9 @@
 • HiPlus Men's Testosterone Booster Power Complex (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Testosterona Natural
-Shilajit del Himalaya
-Potencia Máxima</t>
+    <t xml:space="preserve">Pispa Toro
+Nuara Varonil
+Garra Testo</t>
   </si>
   <si>
     <t>Gladiador: bebida potenciadora sexual masculina</t>
@@ -2429,9 +2431,9 @@
     <t>• Snap Prostate Health &amp; Nitric Oxide Chews (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Gomita Prostática
-Granada Real
-Vigor Nocturno</t>
+    <t xml:space="preserve">Pispa Papi Gummies
+Nuara Granada
+Garra Firme</t>
   </si>
   <si>
     <t>F61</t>
@@ -2451,9 +2453,9 @@
     <t>• Pumpkin Seed Oil + Saw Palmetto Softgel 1000mg (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Aceite de Calabaza
-Ahuyama Dorada
-Vejiga Tranquila</t>
+    <t xml:space="preserve">Pispa Don Calabaza
+Nuara Caudal
+Garra Flujo</t>
   </si>
   <si>
     <t>F60</t>
@@ -2475,9 +2477,9 @@
     <t>• Windboss Suplemento para Hombres (México)</t>
   </si>
   <si>
-    <t xml:space="preserve">Próstata Saludable
-Palma Enana
-Noches Completas</t>
+    <t xml:space="preserve">Pispa Don
+Nuara Plenitud
+Garra Prosta</t>
   </si>
   <si>
     <t>Cerebro y concentración  ·  2 registros</t>
@@ -2501,9 +2503,9 @@
 • Windboss Chicles/Mentas L-Teanina + B12 + B6 (México)</t>
   </si>
   <si>
-    <t xml:space="preserve">Menta Energizante
-Enfoque Puro
-Siempre Despierto</t>
+    <t xml:space="preserve">Pispa Boost
+Nuara Chispa
+Garra Mecha</t>
   </si>
   <si>
     <t>F81</t>
@@ -2521,9 +2523,9 @@
     <t>• Balincer Ginkgo Biloba (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Ginkgo Memoria
-Árbol de la Memoria
-Mente Despierta</t>
+    <t xml:space="preserve">Pispa Focus
+Nuara Memoria
+Garra Mente</t>
   </si>
   <si>
     <t>Articulaciones y huesos  ·  3 registros</t>
@@ -2542,9 +2544,9 @@
     <t>• Airboy Vitamina D3 + K2 (México)</t>
   </si>
   <si>
-    <t xml:space="preserve">Vitamina Solar
-Sol de Mediodía
-Paso Firme</t>
+    <t xml:space="preserve">Pispa Sol Caps
+Nuara Soleada
+Garra Coraza</t>
   </si>
   <si>
     <t>F49</t>
@@ -2565,9 +2567,9 @@
     <t>• Balincer Calcium D3 K2 B12 Complex (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Calcio Articular
-Movimiento Libre
-Rodilla Sana</t>
+    <t xml:space="preserve">Pispa Flex
+Nuara Roble
+Garra Hueso</t>
   </si>
   <si>
     <t>F82</t>
@@ -2587,9 +2589,9 @@
     <t>• LOVING TREE Turmeric Curcumin Gummies (EE. UU.)</t>
   </si>
   <si>
-    <t xml:space="preserve">Cúrcuma Articular
-Oro de la India
-Rodillas Libres</t>
+    <t xml:space="preserve">Pispa Gold
+Nuara Soltura
+Garra Alivio</t>
   </si>
   <si>
     <t>Niños  ·  3 registros</t>
@@ -5486,7 +5488,7 @@
       <xdr:row>27</xdr:row>
       <xdr:rowOff>144750</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="762000" cy="762000"/>
+    <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="21" name="Picture 21">
@@ -5996,7 +5998,7 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>7800</xdr:colOff>
       <xdr:row>11</xdr:row>
-      <xdr:rowOff>36750</xdr:rowOff>
+      <xdr:rowOff>32000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="762000" cy="762000"/>
     <xdr:pic>
@@ -8219,10 +8221,10 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>151500</xdr:rowOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>131250</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="762000" cy="762000"/>
+    <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="16" name="Picture 16">
@@ -8258,8 +8260,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>63750</xdr:rowOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>151500</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -8297,8 +8299,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>57000</xdr:rowOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>63750</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -8336,8 +8338,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>43500</xdr:rowOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>57000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -8375,8 +8377,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>40000</xdr:rowOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>43500</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -8414,8 +8416,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>57000</xdr:rowOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>40000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -8453,7 +8455,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>27</xdr:row>
       <xdr:rowOff>57000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -8492,8 +8494,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>63750</xdr:rowOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>57000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -8531,8 +8533,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>43500</xdr:rowOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>63750</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -8570,8 +8572,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>56999</xdr:rowOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>43500</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -8609,8 +8611,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>43499</xdr:rowOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>56999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -8648,8 +8650,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>70499</xdr:rowOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>43499</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -8687,8 +8689,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>43499</xdr:rowOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>70499</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -8726,8 +8728,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>56999</xdr:rowOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>43499</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -8765,8 +8767,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>39999</xdr:rowOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>56999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -8804,7 +8806,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -8843,7 +8845,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>39</xdr:row>
+      <xdr:row>38</xdr:row>
       <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -8882,7 +8884,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>40</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -8921,7 +8923,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>41</xdr:row>
+      <xdr:row>40</xdr:row>
       <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -8960,8 +8962,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>43</xdr:row>
-      <xdr:rowOff>50249</xdr:rowOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -8999,7 +9001,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>44</xdr:row>
+      <xdr:row>43</xdr:row>
       <xdr:rowOff>50249</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -9038,8 +9040,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>45</xdr:row>
-      <xdr:rowOff>56999</xdr:rowOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>50249</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -9077,8 +9079,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>46</xdr:row>
-      <xdr:rowOff>43499</xdr:rowOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>56999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -9116,8 +9118,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>39999</xdr:rowOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>43499</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -9155,7 +9157,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>48</xdr:row>
+      <xdr:row>47</xdr:row>
       <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -9194,8 +9196,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>50</xdr:row>
-      <xdr:rowOff>50249</xdr:rowOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -9233,8 +9235,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>51</xdr:row>
-      <xdr:rowOff>39999</xdr:rowOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>50249</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -9272,7 +9274,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -9311,8 +9313,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>53</xdr:row>
-      <xdr:rowOff>43499</xdr:rowOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -9350,7 +9352,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>54</xdr:row>
+      <xdr:row>53</xdr:row>
       <xdr:rowOff>43499</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -9389,8 +9391,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>55</xdr:row>
-      <xdr:rowOff>63749</xdr:rowOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>43499</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -9428,8 +9430,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>56</xdr:row>
-      <xdr:rowOff>50249</xdr:rowOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>63749</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -9467,8 +9469,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>57</xdr:row>
-      <xdr:rowOff>63749</xdr:rowOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>50249</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -9506,8 +9508,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>59</xdr:row>
-      <xdr:rowOff>56999</xdr:rowOff>
+      <xdr:row>57</xdr:row>
+      <xdr:rowOff>63749</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -9545,8 +9547,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>60</xdr:row>
-      <xdr:rowOff>39999</xdr:rowOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>56999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -9584,7 +9586,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>61</xdr:row>
+      <xdr:row>60</xdr:row>
       <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -9623,7 +9625,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>62</xdr:row>
+      <xdr:row>61</xdr:row>
       <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -9662,7 +9664,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>63</xdr:row>
+      <xdr:row>62</xdr:row>
       <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -9701,7 +9703,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>64</xdr:row>
+      <xdr:row>63</xdr:row>
       <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -9740,8 +9742,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>65</xdr:row>
-      <xdr:rowOff>56999</xdr:rowOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -9779,8 +9781,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>67</xdr:row>
-      <xdr:rowOff>39999</xdr:rowOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>56999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -9818,7 +9820,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>68</xdr:row>
+      <xdr:row>67</xdr:row>
       <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -9857,7 +9859,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>69</xdr:row>
+      <xdr:row>68</xdr:row>
       <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -9896,7 +9898,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>70</xdr:row>
+      <xdr:row>69</xdr:row>
       <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -9935,8 +9937,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>71</xdr:row>
-      <xdr:rowOff>50249</xdr:rowOff>
+      <xdr:row>70</xdr:row>
+      <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -9974,8 +9976,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>72</xdr:row>
-      <xdr:rowOff>39999</xdr:rowOff>
+      <xdr:row>71</xdr:row>
+      <xdr:rowOff>50249</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -10013,7 +10015,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>74</xdr:row>
+      <xdr:row>72</xdr:row>
       <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -10052,8 +10054,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>75</xdr:row>
-      <xdr:rowOff>50249</xdr:rowOff>
+      <xdr:row>74</xdr:row>
+      <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -10091,8 +10093,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>76</xdr:row>
-      <xdr:rowOff>39999</xdr:rowOff>
+      <xdr:row>75</xdr:row>
+      <xdr:rowOff>50249</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -10130,7 +10132,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>77</xdr:row>
+      <xdr:row>76</xdr:row>
       <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -10169,7 +10171,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>78</xdr:row>
+      <xdr:row>77</xdr:row>
       <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -10208,7 +10210,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>79</xdr:row>
+      <xdr:row>78</xdr:row>
       <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -10247,7 +10249,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>80</xdr:row>
+      <xdr:row>79</xdr:row>
       <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -10286,8 +10288,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>82</xdr:row>
-      <xdr:rowOff>56999</xdr:rowOff>
+      <xdr:row>80</xdr:row>
+      <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -10325,8 +10327,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>83</xdr:row>
-      <xdr:rowOff>39999</xdr:rowOff>
+      <xdr:row>82</xdr:row>
+      <xdr:rowOff>56999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -10364,8 +10366,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>84</xdr:row>
-      <xdr:rowOff>97499</xdr:rowOff>
+      <xdr:row>83</xdr:row>
+      <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -10403,8 +10405,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>85</xdr:row>
-      <xdr:rowOff>50249</xdr:rowOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>97499</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -10442,8 +10444,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>86</xdr:row>
-      <xdr:rowOff>43499</xdr:rowOff>
+      <xdr:row>85</xdr:row>
+      <xdr:rowOff>50249</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -10481,8 +10483,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>87</xdr:row>
-      <xdr:rowOff>39999</xdr:rowOff>
+      <xdr:row>86</xdr:row>
+      <xdr:rowOff>43499</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -10520,8 +10522,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>89</xdr:row>
-      <xdr:rowOff>83999</xdr:rowOff>
+      <xdr:row>87</xdr:row>
+      <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -10559,8 +10561,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>90</xdr:row>
-      <xdr:rowOff>43499</xdr:rowOff>
+      <xdr:row>89</xdr:row>
+      <xdr:rowOff>83999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -10598,8 +10600,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>91</xdr:row>
-      <xdr:rowOff>39999</xdr:rowOff>
+      <xdr:row>90</xdr:row>
+      <xdr:rowOff>43499</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -10637,8 +10639,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>94</xdr:row>
-      <xdr:rowOff>63749</xdr:rowOff>
+      <xdr:row>91</xdr:row>
+      <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -10676,8 +10678,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>95</xdr:row>
-      <xdr:rowOff>39999</xdr:rowOff>
+      <xdr:row>92</xdr:row>
+      <xdr:rowOff>151499</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -10715,8 +10717,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>96</xdr:row>
-      <xdr:rowOff>39999</xdr:rowOff>
+      <xdr:row>94</xdr:row>
+      <xdr:rowOff>63749</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -10754,7 +10756,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>98</xdr:row>
+      <xdr:row>95</xdr:row>
       <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -10793,7 +10795,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>99</xdr:row>
+      <xdr:row>96</xdr:row>
       <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -10832,7 +10834,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>101</xdr:row>
+      <xdr:row>98</xdr:row>
       <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -10871,7 +10873,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>102</xdr:row>
+      <xdr:row>99</xdr:row>
       <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -10910,7 +10912,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>103</xdr:row>
+      <xdr:row>101</xdr:row>
       <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -10949,8 +10951,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>105</xdr:row>
-      <xdr:rowOff>43499</xdr:rowOff>
+      <xdr:row>102</xdr:row>
+      <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -10988,7 +10990,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>107</xdr:row>
+      <xdr:row>103</xdr:row>
       <xdr:rowOff>39999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
@@ -11027,8 +11029,8 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>15600</xdr:colOff>
-      <xdr:row>109</xdr:row>
-      <xdr:rowOff>39999</xdr:rowOff>
+      <xdr:row>105</xdr:row>
+      <xdr:rowOff>43499</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1676400" cy="942975"/>
     <xdr:pic>
@@ -11046,6 +11048,123 @@
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId88" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>15600</xdr:colOff>
+      <xdr:row>106</xdr:row>
+      <xdr:rowOff>83999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1676400" cy="942975"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="89" name="Picture 89">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId89" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>15600</xdr:colOff>
+      <xdr:row>107</xdr:row>
+      <xdr:rowOff>39999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1676400" cy="942975"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="90" name="Picture 90">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId90" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>15600</xdr:colOff>
+      <xdr:row>109</xdr:row>
+      <xdr:rowOff>39999</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1676400" cy="942975"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="91" name="Picture 91">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId91" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -12008,7 +12127,7 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>7800</xdr:colOff>
       <xdr:row>34</xdr:row>
-      <xdr:rowOff>36749</xdr:rowOff>
+      <xdr:rowOff>31999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="762000" cy="762000"/>
     <xdr:pic>
@@ -12047,7 +12166,7 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>7800</xdr:colOff>
       <xdr:row>35</xdr:row>
-      <xdr:rowOff>36749</xdr:rowOff>
+      <xdr:rowOff>31999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="762000" cy="762000"/>
     <xdr:pic>
@@ -12086,7 +12205,7 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>7800</xdr:colOff>
       <xdr:row>36</xdr:row>
-      <xdr:rowOff>36749</xdr:rowOff>
+      <xdr:rowOff>31999</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="762000" cy="762000"/>
     <xdr:pic>
@@ -18884,7 +19003,7 @@
       <c r="K11" s="26"/>
       <c r="L11" s="26"/>
     </row>
-    <row r="12" ht="73.5" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="12" ht="64" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="6"/>
       <c r="B12" s="7" t="s">
         <v>1116</v>
@@ -26141,7 +26260,7 @@
       <c r="K34" s="26"/>
       <c r="L34" s="26"/>
     </row>
-    <row r="35" ht="73.5" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="35" ht="64" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="6"/>
       <c r="B35" s="7" t="s">
         <v>748</v>
@@ -26177,7 +26296,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="36" ht="73.5" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="36" ht="64" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="14"/>
       <c r="B36" s="15" t="s">
         <v>751</v>
@@ -26211,7 +26330,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="37" ht="73.5" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="37" ht="64" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="6"/>
       <c r="B37" s="7" t="s">
         <v>754</v>

</xml_diff>